<commit_message>
Refresh players export — 40 plays snapshot
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/share/Etienne-Players.xlsx
+++ b/public/share/Etienne-Players.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -642,16 +642,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>@salfajji</t>
+          <t>@zabzyy</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>salfajji</t>
+          <t>zabzyy</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>850</v>
+        <v>1031</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-03  20:13</t>
+          <t>2026-05-05  16:07</t>
         </is>
       </c>
     </row>
@@ -670,16 +670,16 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>@icu96_</t>
+          <t>@noor11_09</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>icu96_</t>
+          <t>noor11_09</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>832</v>
+        <v>965</v>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>2026-05-03  18:32</t>
+          <t>2026-05-04  23:22</t>
         </is>
       </c>
     </row>
@@ -698,25 +698,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>@eng_menawer</t>
+          <t>@abdullahaljarki</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>eng_menawer</t>
+          <t>abdullahaljarki</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>813</v>
+        <v>947</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Etienne</t>
+          <t>River</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-03  18:52</t>
+          <t>2026-05-05  17:54</t>
         </is>
       </c>
     </row>
@@ -726,16 +726,16 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>@farahpunzel</t>
+          <t>@farahmorad</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>farahpunzel</t>
+          <t>farahmorad</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>799</v>
+        <v>895</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2026-05-04  12:23</t>
+          <t>2026-05-05  07:48</t>
         </is>
       </c>
     </row>
@@ -754,16 +754,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>@bbritto99</t>
+          <t>@salfajji</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>bbritto99</t>
+          <t>salfajji</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>798</v>
+        <v>850</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>2026-05-04  00:06</t>
+          <t>2026-05-03  20:13</t>
         </is>
       </c>
     </row>
@@ -782,16 +782,16 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>@w1nb</t>
+          <t>@icu96_</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>w1nb</t>
+          <t>icu96_</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>773</v>
+        <v>832</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>2026-05-04  06:05</t>
+          <t>2026-05-03  18:32</t>
         </is>
       </c>
     </row>
@@ -810,25 +810,25 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>@aminaonthemat</t>
+          <t>@tipicokwt</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>aminaonthemat</t>
+          <t>tipicokwt</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>750</v>
+        <v>815</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wild Cotton</t>
+          <t>River</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>2026-05-03  19:16</t>
+          <t>2026-05-05  13:54</t>
         </is>
       </c>
     </row>
@@ -838,25 +838,25 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>@kjalabdul</t>
+          <t>@eng_menawer</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>kjalabdul</t>
+          <t>eng_menawer</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>722</v>
+        <v>813</v>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Linen</t>
+          <t>Etienne</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>2026-05-03  21:44</t>
+          <t>2026-05-03  18:52</t>
         </is>
       </c>
     </row>
@@ -866,25 +866,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>@badoraaals</t>
+          <t>@manayel.ahmad</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>badoraaals</t>
+          <t>manayel.ahmad</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>697</v>
+        <v>809</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Etienne</t>
+          <t>Wild Cotton</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>2026-05-03  21:06</t>
+          <t>2026-05-05  15:55</t>
         </is>
       </c>
     </row>
@@ -894,25 +894,25 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>@m_alwazzan88</t>
+          <t>@farahpunzel</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>m_alwazzan88</t>
+          <t>farahpunzel</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>684</v>
+        <v>799</v>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Linen</t>
+          <t>Etienne</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>2026-05-03  22:57</t>
+          <t>2026-05-04  12:23</t>
         </is>
       </c>
     </row>
@@ -922,16 +922,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>@ghazitark</t>
+          <t>@bbritto99</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ghazitark</t>
+          <t>bbritto99</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>627</v>
+        <v>798</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>2026-05-03  22:45</t>
+          <t>2026-05-04  00:06</t>
         </is>
       </c>
     </row>
@@ -950,16 +950,16 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>@sonanddark</t>
+          <t>@w1nb</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>sonanddark</t>
+          <t>w1nb</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>590</v>
+        <v>773</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>2026-05-03  18:37</t>
+          <t>2026-05-04  06:05</t>
         </is>
       </c>
     </row>
@@ -978,25 +978,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>@falnaqeeb</t>
+          <t>@haya</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>falnaqeeb</t>
+          <t>haya</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>590</v>
+        <v>769</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>River</t>
+          <t>Etienne</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>2026-05-03  20:12</t>
+          <t>2026-05-04  23:02</t>
         </is>
       </c>
     </row>
@@ -1006,16 +1006,16 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>@rydeenn</t>
+          <t>@qemlas</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>rydeenn</t>
+          <t>qemlas</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>516</v>
+        <v>762</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>2026-05-03  18:43</t>
+          <t>2026-05-05  15:38</t>
         </is>
       </c>
     </row>
@@ -1034,25 +1034,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>@aminaxsalim</t>
+          <t>@aminaonthemat</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>aminaxsalim</t>
+          <t>aminaonthemat</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>488</v>
+        <v>750</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Etienne</t>
+          <t>Wild Cotton</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>2026-05-03  19:13</t>
+          <t>2026-05-03  19:16</t>
         </is>
       </c>
     </row>
@@ -1062,25 +1062,25 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>@mfalhaaa</t>
+          <t>@kjalabdul</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>mfalhaaa</t>
+          <t>kjalabdul</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>453</v>
+        <v>722</v>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Etienne</t>
+          <t>Linen</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>2026-05-03  23:27</t>
+          <t>2026-05-03  21:44</t>
         </is>
       </c>
     </row>
@@ -1090,16 +1090,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>@salemalharan</t>
+          <t>@badoraaals</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>salemalharan</t>
+          <t>badoraaals</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>442</v>
+        <v>697</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>2026-05-04  02:55</t>
+          <t>2026-05-03  21:06</t>
         </is>
       </c>
     </row>
@@ -1118,25 +1118,25 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>@v97o0</t>
+          <t>@m_alwazzan88</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>v97o0</t>
+          <t>m_alwazzan88</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>382</v>
+        <v>684</v>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Etienne</t>
+          <t>Linen</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>2026-05-04  06:03</t>
+          <t>2026-05-03  22:57</t>
         </is>
       </c>
     </row>
@@ -1146,25 +1146,473 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>@ghazitark</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ghazitark</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>627</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-03  22:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>@jojo_mahmd965</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>jojo_mahmd965</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>593</v>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-05  16:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>@sonanddark</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>sonanddark</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>590</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-03  18:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>@falnaqeeb</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>falnaqeeb</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>590</v>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>River</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-03  20:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>@has.2002</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>has.2002</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>528</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-04  16:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>@rydeenn</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>rydeenn</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>516</v>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-03  18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>@haalkharji</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>haalkharji</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>513</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-05  03:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>@shalhouli</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>shalhouli</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>511</v>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-04  23:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>@9agerrr</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>9agerrr</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>493</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-04  14:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>@aminaxsalim</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>aminaxsalim</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>488</v>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-03  19:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>@lolo</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>lolo</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>481</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-05  16:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>@mfalhaaa</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>mfalhaaa</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>453</v>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-03  23:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>@salemalharan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>salemalharan</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>442</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-04  02:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>@Elaf_kossale</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>elaf_kossale</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>432</v>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-05  21:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>@v97o0</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>v97o0</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>382</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-04  06:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
           <t>@Jaljaiedan</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>jaljaiedan</t>
         </is>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D40" s="5" t="n">
         <v>359</v>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Etienne</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Etienne</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>2026-05-03  20:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>@sa.alabdali</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>sa.alabdali</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>253</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Wild Cotton</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-05  05:24</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1653,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -1237,7 +1685,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>359</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6">
@@ -1247,7 +1695,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>750</v>
+        <v>720</v>
       </c>
     </row>
     <row r="7">
@@ -1258,7 +1706,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-04  13:42  Kuwait</t>
+          <t>2026-05-05  22:11  Kuwait</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1729,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11">
@@ -1291,27 +1739,27 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Linen</t>
+          <t>River</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>River</t>
+          <t>Linen</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>